<commit_message>
Add Performance DO Return KPI formatting
</commit_message>
<xml_diff>
--- a/FORMATTING.xlsx
+++ b/FORMATTING.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SAPX\Data Analisis\RealKPI vs NoteUserKPI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D04C580D-A4B3-49A1-832E-7371E1BB3F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E1808C-49BA-4A8D-8317-E38D4E151D48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" xr2:uid="{87F6102B-F5E6-4225-820A-6C7AB19EA969}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="26">
   <si>
     <t>OS Outgoing Return</t>
   </si>
@@ -100,19 +100,28 @@
   </si>
   <si>
     <t>KPI Indices</t>
+  </si>
+  <si>
+    <t>Performance DO Return</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -135,11 +144,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -454,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{722029E8-6599-4819-84F1-997C754C52FE}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="43.6640625" bestFit="1" customWidth="1"/>
@@ -687,6 +697,20 @@
         <v>20</v>
       </c>
     </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A17" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>